<commit_message>
Merge main into nr-doc-core-encounter, résout conflit change_notes.md
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com> 807e5653b25ff2bf511a1b2f95a4cf280e6899a0
</commit_message>
<xml_diff>
--- a/nr-doc-core-encounter/ig/CodeSystem-fr-core-cs-mode-validation-identity.xlsx
+++ b/nr-doc-core-encounter/ig/CodeSystem-fr-core-cs-mode-validation-identity.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="75">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-10-13T09:01:17+00:00</t>
+    <t>2026-10-13T11:52:39+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -126,7 +126,7 @@
     <t>Count</t>
   </si>
   <si>
-    <t>14</t>
+    <t>15</t>
   </si>
   <si>
     <t>Level</t>
@@ -144,91 +144,100 @@
     <t>1</t>
   </si>
   <si>
+    <t>CN</t>
+  </si>
+  <si>
+    <t>Carte nationale d'identité</t>
+  </si>
+  <si>
+    <t>PA</t>
+  </si>
+  <si>
+    <t>Passeport</t>
+  </si>
+  <si>
+    <t>CS</t>
+  </si>
+  <si>
+    <t>Carte de séjour</t>
+  </si>
+  <si>
+    <t>Carte de séjour ou titre de séjour</t>
+  </si>
+  <si>
+    <t>eCN</t>
+  </si>
+  <si>
+    <t>e-carte d'identité</t>
+  </si>
+  <si>
+    <t>IN</t>
+  </si>
+  <si>
+    <t>Identité Numérique La Poste</t>
+  </si>
+  <si>
+    <t>AV</t>
+  </si>
+  <si>
+    <t>Application Carte Vitale</t>
+  </si>
+  <si>
+    <t>LECV</t>
+  </si>
+  <si>
+    <t>Livret de famille, accompagné de la carte Vitale avec photographie</t>
+  </si>
+  <si>
     <t>AN</t>
   </si>
   <si>
     <t>Extrait d'acte de naissance</t>
   </si>
   <si>
+    <t>LE</t>
+  </si>
+  <si>
+    <t>Livret de famille des parents</t>
+  </si>
+  <si>
     <t>CC</t>
   </si>
   <si>
     <t>Carnet de circulation</t>
   </si>
   <si>
-    <t>CE</t>
-  </si>
-  <si>
-    <t>Carte Européenne</t>
-  </si>
-  <si>
-    <t>CN</t>
-  </si>
-  <si>
-    <t>Carte nationale d'identité</t>
-  </si>
-  <si>
-    <t>LE</t>
-  </si>
-  <si>
-    <t>Livret de famille</t>
-  </si>
-  <si>
-    <t>PA</t>
-  </si>
-  <si>
-    <t>Passeport</t>
+    <t>Carnet de circulation pour étranger mineur</t>
+  </si>
+  <si>
+    <t>CIMS</t>
+  </si>
+  <si>
+    <t>Carte d'identité professionnelle multiservices (CIMS)</t>
+  </si>
+  <si>
+    <t>ANCV</t>
+  </si>
+  <si>
+    <t>Extrait d'acte de naissance, accompagné de la carte Vitale avec photographie</t>
+  </si>
+  <si>
+    <t>IE</t>
+  </si>
+  <si>
+    <t>Identification électronique EIDAS</t>
+  </si>
+  <si>
+    <t>CM</t>
+  </si>
+  <si>
+    <t>Carte militaire</t>
   </si>
   <si>
     <t>PC</t>
   </si>
   <si>
     <t>Permis de conduire</t>
-  </si>
-  <si>
-    <t>TC</t>
-  </si>
-  <si>
-    <t>Tiers de confiance</t>
-  </si>
-  <si>
-    <t>AC</t>
-  </si>
-  <si>
-    <t>Acte de naissance + Carte vitale avec photo</t>
-  </si>
-  <si>
-    <t>AV</t>
-  </si>
-  <si>
-    <t>Application Carte Vitale</t>
-  </si>
-  <si>
-    <t>CS</t>
-  </si>
-  <si>
-    <t>Carte de séjour</t>
-  </si>
-  <si>
-    <t>Carte de séjour ou titre de séjour</t>
-  </si>
-  <si>
-    <t>IE</t>
-  </si>
-  <si>
-    <t>Identification électronique EIDAS</t>
-  </si>
-  <si>
-    <t>DC</t>
-  </si>
-  <si>
-    <t>Document de Circulation pour étranger mineur</t>
-  </si>
-  <si>
-    <t>CM</t>
-  </si>
-  <si>
-    <t>Carte militaire</t>
   </si>
 </sst>
 </file>
@@ -546,7 +555,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -602,7 +611,7 @@
         <v>48</v>
       </c>
       <c r="D4" t="s" s="2">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5">
@@ -610,13 +619,13 @@
         <v>42</v>
       </c>
       <c r="B5" t="s" s="2">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C5" t="s" s="2">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D5" t="s" s="2">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6">
@@ -624,13 +633,13 @@
         <v>42</v>
       </c>
       <c r="B6" t="s" s="2">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C6" t="s" s="2">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D6" t="s" s="2">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7">
@@ -638,13 +647,13 @@
         <v>42</v>
       </c>
       <c r="B7" t="s" s="2">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C7" t="s" s="2">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D7" t="s" s="2">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8">
@@ -652,13 +661,13 @@
         <v>42</v>
       </c>
       <c r="B8" t="s" s="2">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C8" t="s" s="2">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D8" t="s" s="2">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="9">
@@ -666,13 +675,13 @@
         <v>42</v>
       </c>
       <c r="B9" t="s" s="2">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C9" t="s" s="2">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D9" t="s" s="2">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10">
@@ -680,13 +689,13 @@
         <v>42</v>
       </c>
       <c r="B10" t="s" s="2">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C10" t="s" s="2">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D10" t="s" s="2">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="11">
@@ -694,13 +703,13 @@
         <v>42</v>
       </c>
       <c r="B11" t="s" s="2">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C11" t="s" s="2">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D11" t="s" s="2">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="12">
@@ -708,13 +717,13 @@
         <v>42</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C12" t="s" s="2">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D12" t="s" s="2">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="13">
@@ -722,13 +731,13 @@
         <v>42</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C13" t="s" s="2">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D13" t="s" s="2">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="14">
@@ -736,13 +745,13 @@
         <v>42</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C14" t="s" s="2">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D14" t="s" s="2">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="15">
@@ -750,13 +759,27 @@
         <v>42</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C15" t="s" s="2">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D15" t="s" s="2">
-        <v>71</v>
+        <v>72</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s" s="2">
+        <v>42</v>
+      </c>
+      <c r="B16" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="C16" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="D16" t="s" s="2">
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>